<commit_message>
Updated UGA_grids_kan model - 2025-12-22 19:23
</commit_message>
<xml_diff>
--- a/VerveStacks_UGA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_UGA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_UGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F65A617E-77A7-4C64-8A16-4407585105D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1B43B8F5-C43C-4705-ABC2-EA91ECEC9E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5115,7 +5115,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66054BBE-3569-4EE2-84D4-C66306D36898}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AA96646-8BB7-456F-950B-C66324B789E2}">
   <dimension ref="B9:L71"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24597,7 +24597,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F224C5C3-F5D0-4A61-AB13-5F9085448A94}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7C33D9-FA63-468B-9593-41BCFD898332}">
   <dimension ref="B9:H71"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>